<commit_message>
Map each beach fill and check its extent against CoastSat
Add placement dates with sources, a figure of each fill's reported limits
over the model domains, single-fill maps and a paper figure with a
locator, and a summary table. Check each footprint against CoastSat
shorelines before and after placement, with animations. The 2026 Avon
and Buxton fills appear on the maps but stay out of the model.
</commit_message>
<xml_diff>
--- a/data/hatteras_init/4-mgmt-forcing/nourishment/datasets/Hatteras_BN_data.xlsx
+++ b/data/hatteras_init/4-mgmt-forcing/nourishment/datasets/Hatteras_BN_data.xlsx
@@ -12,9 +12,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd hh:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="4">
     <font>
@@ -2779,7 +2778,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="n">
+      <c r="A30" s="0" t="n">
         <v>4274</v>
       </c>
       <c r="B30" s="6" t="n">
@@ -2788,79 +2787,79 @@
       <c r="C30" s="6" t="n">
         <v>44979.79597359954</v>
       </c>
-      <c r="D30" t="n">
+      <c r="D30" s="0" t="n">
         <v>307</v>
       </c>
-      <c r="E30" t="inlineStr">
+      <c r="E30" s="0" t="inlineStr">
         <is>
           <t>NC / Buxton</t>
         </is>
       </c>
-      <c r="F30" t="inlineStr">
+      <c r="F30" s="0" t="inlineStr">
         <is>
           <t>NC</t>
         </is>
       </c>
-      <c r="G30" t="inlineStr">
+      <c r="G30" s="0" t="inlineStr">
         <is>
           <t>Buxton</t>
         </is>
       </c>
-      <c r="H30" t="n">
+      <c r="H30" s="0" t="n">
         <v>35.282537</v>
       </c>
-      <c r="I30" t="n">
+      <c r="I30" s="0" t="n">
         <v>-75.515334</v>
       </c>
-      <c r="J30" t="n">
+      <c r="J30" s="0" t="n">
         <v>2022</v>
       </c>
-      <c r="K30" t="inlineStr">
+      <c r="K30" s="0" t="inlineStr">
         <is>
           <t>Local</t>
         </is>
       </c>
-      <c r="L30" t="inlineStr">
+      <c r="L30" s="0" t="inlineStr">
         <is>
           <t>Shore Protection</t>
         </is>
       </c>
-      <c r="M30" t="n">
+      <c r="M30" s="0" t="n">
         <v>15312</v>
       </c>
-      <c r="N30" t="n">
+      <c r="N30" s="0" t="n">
         <v>1200000</v>
       </c>
-      <c r="O30" t="n">
+      <c r="O30" s="0" t="n">
         <v>18106674</v>
       </c>
-      <c r="P30" t="n">
+      <c r="P30" s="0" t="n">
         <v>292.7</v>
       </c>
-      <c r="Q30" t="n">
+      <c r="Q30" s="0" t="n">
         <v>19449054.68</v>
       </c>
-      <c r="R30" t="n">
+      <c r="R30" s="0" t="n">
         <v>15.09</v>
       </c>
-      <c r="S30" t="n">
+      <c r="S30" s="0" t="n">
         <v>16.21</v>
       </c>
-      <c r="T30" t="n">
+      <c r="T30" s="0" t="n">
         <v>78.37</v>
       </c>
-      <c r="U30" t="n">
+      <c r="U30" s="0" t="n">
         <v>2024</v>
       </c>
-      <c r="V30" t="n">
+      <c r="V30" s="0" t="n">
         <v>314.4</v>
       </c>
-      <c r="W30" t="inlineStr">
+      <c r="W30" s="0" t="inlineStr">
         <is>
           <t>Copied from the source dataset (id 4274) by H. Henry 2026-10-02, values unchanged. The source's sourceComment pointed to the 2018 article on the 2017-18 project (https://outerbanksvoice.com/2018/03/01/delayed-buxton-beach-nourishment-project-is-finally-done/); replaced with a 2022 source. Placed 2022-06-30 to 2022-08-16, Haulover Day Use Area to the lighthouse groin field.</t>
         </is>
       </c>
-      <c r="X30" t="inlineStr">
+      <c r="X30" s="0" t="inlineStr">
         <is>
           <t>https://content.govdelivery.com/accounts/NCDARECOUNTY/bulletins/3285a2f</t>
         </is>
@@ -2953,68 +2952,68 @@
       <c r="C32" s="6" t="n">
         <v>46297</v>
       </c>
-      <c r="F32" t="inlineStr">
+      <c r="F32" s="0" t="inlineStr">
         <is>
           <t>NC</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr">
+      <c r="G32" s="0" t="inlineStr">
         <is>
           <t>Avon</t>
         </is>
       </c>
-      <c r="H32" t="n">
+      <c r="H32" s="0" t="n">
         <v>35.3385765</v>
       </c>
-      <c r="I32" t="n">
+      <c r="I32" s="0" t="n">
         <v>-75.5038756</v>
       </c>
-      <c r="J32" t="n">
+      <c r="J32" s="0" t="n">
         <v>2026</v>
       </c>
-      <c r="K32" t="inlineStr">
+      <c r="K32" s="0" t="inlineStr">
         <is>
           <t>Local</t>
         </is>
       </c>
-      <c r="L32" t="inlineStr">
+      <c r="L32" s="0" t="inlineStr">
         <is>
           <t>Shore Protection</t>
         </is>
       </c>
-      <c r="M32" t="n">
+      <c r="M32" s="0" t="n">
         <v>5280</v>
       </c>
-      <c r="N32" t="n">
+      <c r="N32" s="0" t="n">
         <v>375000</v>
       </c>
-      <c r="O32" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q32" t="n">
-        <v>0</v>
-      </c>
-      <c r="R32" t="n">
-        <v>0</v>
-      </c>
-      <c r="S32" t="n">
-        <v>0</v>
-      </c>
-      <c r="T32" t="n">
+      <c r="O32" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q32" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="R32" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="S32" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="T32" s="0" t="n">
         <v>71.02</v>
       </c>
-      <c r="U32" t="n">
+      <c r="U32" s="0" t="n">
         <v>2024</v>
       </c>
-      <c r="V32" t="n">
+      <c r="V32" s="0" t="n">
         <v>314.4</v>
       </c>
-      <c r="W32" t="inlineStr">
-        <is>
-          <t>Added by H. Henry 2026-10-02; not yet in the national database. Placed 2026-05-27 to 2026-06-25, from just south of Avon Pier to the south village limit near Greenwood Place, ~1 mi (extent from one secondary source). Cost not reported separately (Avon + Buxton 2026 combined ~$45 M), so cost fields are 0. Lat/long copied from id 6469.</t>
-        </is>
-      </c>
-      <c r="X32" t="inlineStr">
+      <c r="W32" s="0" t="inlineStr">
+        <is>
+          <t>Added by H. Henry 2026-10-02; not yet in the national database. Placed 2026-05-28 to 2026-06-25 (planned start 05-27), from just south of Avon Pier to the south village limit near Greenwood Place, ~1 mi (extent from one secondary source). Cost not reported separately (Avon + Buxton 2026 combined ~$45 M), so cost fields are 0. Lat/long copied from id 6469.</t>
+        </is>
+      </c>
+      <c r="X32" s="0" t="inlineStr">
         <is>
           <t>https://www.outerbanksvoice.com/2026/05/26/avon-beach-nourishment-project-expected-to-begin-on-wednesday-may-27/ ; https://www.usbeachlife.com/avon-nc/beach-erosion</t>
         </is>
@@ -3027,76 +3026,76 @@
       <c r="C33" s="6" t="n">
         <v>46297</v>
       </c>
-      <c r="D33" t="n">
+      <c r="D33" s="0" t="n">
         <v>307</v>
       </c>
-      <c r="E33" t="inlineStr">
+      <c r="E33" s="0" t="inlineStr">
         <is>
           <t>NC / Buxton</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr">
+      <c r="F33" s="0" t="inlineStr">
         <is>
           <t>NC</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr">
+      <c r="G33" s="0" t="inlineStr">
         <is>
           <t>Buxton</t>
         </is>
       </c>
-      <c r="H33" t="n">
+      <c r="H33" s="0" t="n">
         <v>35.282537</v>
       </c>
-      <c r="I33" t="n">
+      <c r="I33" s="0" t="n">
         <v>-75.515334</v>
       </c>
-      <c r="J33" t="n">
+      <c r="J33" s="0" t="n">
         <v>2026</v>
       </c>
-      <c r="K33" t="inlineStr">
+      <c r="K33" s="0" t="inlineStr">
         <is>
           <t>Local</t>
         </is>
       </c>
-      <c r="L33" t="inlineStr">
+      <c r="L33" s="0" t="inlineStr">
         <is>
           <t>Shore Protection</t>
         </is>
       </c>
-      <c r="M33" t="n">
+      <c r="M33" s="0" t="n">
         <v>15312</v>
       </c>
-      <c r="N33" t="n">
+      <c r="N33" s="0" t="n">
         <v>2000000</v>
       </c>
-      <c r="O33" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q33" t="n">
-        <v>0</v>
-      </c>
-      <c r="R33" t="n">
-        <v>0</v>
-      </c>
-      <c r="S33" t="n">
-        <v>0</v>
-      </c>
-      <c r="T33" t="n">
+      <c r="O33" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q33" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="R33" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="S33" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="T33" s="0" t="n">
         <v>130.62</v>
       </c>
-      <c r="U33" t="n">
+      <c r="U33" s="0" t="n">
         <v>2024</v>
       </c>
-      <c r="V33" t="n">
+      <c r="V33" s="0" t="n">
         <v>314.4</v>
       </c>
-      <c r="W33" t="inlineStr">
+      <c r="W33" s="0" t="inlineStr">
         <is>
           <t>Added by H. Henry 2026-10-02; not yet in the national database. PLANNED volume, not as-built: pumping began 2026-07-31, ~1.5 M cy (75%) by 2026-09-16, completion expected early Oct 2026 - check the final volume. Base design 1,351,616 cy, raised to 2 M on 2026-05-11 with FEMA funds for Potential Tropical Cyclone Eight (2024). Haulover Day Use Area to the lighthouse groin field, ~2.9 mi. Cost not reported separately (Avon + Buxton 2026 combined ~$45 M), so cost fields are 0. Lat/long copied from id 4274.</t>
         </is>
       </c>
-      <c r="X33" t="inlineStr">
+      <c r="X33" s="0" t="inlineStr">
         <is>
           <t>https://www.outerbanksvoice.com/2026/09/17/latest-update-on-buxton-beach-nourishment-and-groin-repair/ ; https://islandfreepress.org/blog/avon-and-buxton-beach-nourishment-faqs-2026-edition/</t>
         </is>

</xml_diff>